<commit_message>
Atualizar LISTA.xlsx pelo Azure DevOps
</commit_message>
<xml_diff>
--- a/LISTA.xlsx
+++ b/LISTA.xlsx
@@ -1558,7 +1558,7 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>QA Pile</t>
+          <t>Validating</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -2214,7 +2214,7 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Validating</t>
+          <t>Rework</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
@@ -3420,7 +3420,7 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>QA Pile</t>
+          <t>Rework</t>
         </is>
       </c>
       <c r="H56" s="2" t="n">
@@ -3712,7 +3712,11 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="N61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>V.01 R.05</t>
+        </is>
+      </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
           <t>Promob\Wonder Squad</t>
@@ -3720,7 +3724,7 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Promob</t>
+          <t>Promob\2026\Q3</t>
         </is>
       </c>
       <c r="Q61" s="2" t="n">
@@ -3765,7 +3769,11 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>V.01 R.05</t>
+        </is>
+      </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
           <t>Promob\Wonder Squad</t>
@@ -3773,7 +3781,7 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Promob</t>
+          <t>Promob\2026\Q3</t>
         </is>
       </c>
       <c r="Q62" s="2" t="n">
@@ -3814,7 +3822,11 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="N63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>V.01 R.05</t>
+        </is>
+      </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
           <t>Promob\Wonder Squad</t>
@@ -3822,7 +3834,7 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Promob</t>
+          <t>Promob\2026\Q3</t>
         </is>
       </c>
       <c r="Q63" s="2" t="n">
@@ -3863,7 +3875,11 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="N64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>V.01 R.05</t>
+        </is>
+      </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
           <t>Promob\Wonder Squad</t>
@@ -3871,7 +3887,7 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Promob</t>
+          <t>Promob\2026\Q3</t>
         </is>
       </c>
       <c r="Q64" s="2" t="n">
@@ -3893,7 +3909,7 @@
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="H65" s="2" t="n">
@@ -4195,7 +4211,7 @@
         </is>
       </c>
       <c r="H71" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4533,7 @@
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>QA Pile</t>
         </is>
       </c>
       <c r="H77" s="2" t="n">
@@ -4807,7 +4823,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>ZendeskTicket</t>
+          <t>V.01 R.10; ZendeskTicket</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr">
@@ -20224,7 +20240,7 @@
       </c>
       <c r="N379" s="2" t="inlineStr">
         <is>
-          <t>e-desk</t>
+          <t>e-desk; V.01 R.05</t>
         </is>
       </c>
       <c r="O379" s="2" t="inlineStr">
@@ -20234,7 +20250,7 @@
       </c>
       <c r="P379" s="2" t="inlineStr">
         <is>
-          <t>Promob</t>
+          <t>Promob\2026\Q3</t>
         </is>
       </c>
       <c r="Q379" s="2" t="n">
@@ -35904,7 +35920,11 @@
       <c r="K681" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="L681" s="2" t="inlineStr"/>
+      <c r="L681" s="2" t="inlineStr">
+        <is>
+          <t>Guilherme Fernandes da Silva</t>
+        </is>
+      </c>
       <c r="M681" s="2" t="inlineStr">
         <is>
           <t>User Story</t>
@@ -36002,7 +36022,11 @@
       <c r="K683" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L683" s="2" t="inlineStr"/>
+      <c r="L683" s="2" t="inlineStr">
+        <is>
+          <t>Guilherme Fernandes da Silva</t>
+        </is>
+      </c>
       <c r="M683" s="2" t="inlineStr">
         <is>
           <t>User Story</t>
@@ -36407,7 +36431,7 @@
       <c r="F691" s="2" t="inlineStr"/>
       <c r="G691" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="H691" s="2" t="n">
@@ -36717,7 +36741,7 @@
       </c>
       <c r="G697" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="H697" s="2" t="n">
@@ -37074,7 +37098,7 @@
       <c r="F704" s="2" t="inlineStr"/>
       <c r="G704" s="2" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H704" s="2" t="n">
@@ -37533,7 +37557,7 @@
       <c r="F713" s="2" t="inlineStr"/>
       <c r="G713" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H713" s="2" t="n">
@@ -37544,7 +37568,11 @@
         <v>2</v>
       </c>
       <c r="K713" s="2" t="inlineStr"/>
-      <c r="L713" s="2" t="inlineStr"/>
+      <c r="L713" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Suiani dos Santos Babinski</t>
+        </is>
+      </c>
       <c r="M713" s="2" t="inlineStr">
         <is>
           <t>Feature</t>
@@ -37580,7 +37608,7 @@
       </c>
       <c r="G714" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H714" s="2" t="n">
@@ -37591,7 +37619,11 @@
       <c r="K714" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L714" s="2" t="inlineStr"/>
+      <c r="L714" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Suiani dos Santos Babinski</t>
+        </is>
+      </c>
       <c r="M714" s="2" t="inlineStr">
         <is>
           <t>User Story</t>

</xml_diff>